<commit_message>
update co2 comm geo
</commit_message>
<xml_diff>
--- a/VerveStacks_POL_grids_kan50/SubRES_Tmpl/SubRES_Data_Centers_Trans.xlsx
+++ b/VerveStacks_POL_grids_kan50/SubRES_Tmpl/SubRES_Data_Centers_Trans.xlsx
@@ -537,7 +537,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>e_Warsaw_POL</t>
+          <t>e_Zabki_POL</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -560,19 +560,19 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>e_Sosnowiec_POL</t>
+          <t>e_Giszowiec_POL</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>grid node -- way/183945016-220 (Katowice, 19 km)</t>
+          <t>grid node -- PL55-220 (Katowice, 8 km)</t>
         </is>
       </c>
       <c r="C3" t="n">
         <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>321</v>
+        <v>327</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -593,7 +593,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>e_Poznan_POL</t>
+          <t>e_Swarzedz_POL</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -629,7 +629,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>grid node -- way/87667718-220 (Krakow, 12 km)</t>
+          <t>grid node -- way/189501431-400 (Krakow, 13 km)</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -673,7 +673,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>e_Gdansk_POL</t>
+          <t>e_Rumia_POL</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -688,12 +688,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>e_Lomza_POL</t>
+          <t>e_Otwock_POL</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>grid node -- way/121656686-220 (Lomza, 31 km)</t>
+          <t>grid node -- PL26-400 (Warsaw, 53 km)</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -703,12 +703,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>e_Katowice_POL</t>
+          <t>e_PiotrkowTrybunalsk_POL</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>grid node -- way/40946790-220 (Katowice, 19 km)</t>
+          <t>grid node -- way/293484891-400 (Piotrkow Trybunalski, 26 km)</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -718,16 +718,16 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>e_Gliwice_POL</t>
+          <t>e_Bialystok_POL</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>grid node -- way/293489607-400 (Katowice, 21 km)</t>
+          <t>grid node -- PL17-400 (Bialystok, 26 km)</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -743,16 +743,16 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>e_PiotrkowTrybunalsk_POL</t>
+          <t>e_Torun_POL</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>grid node -- way/170316833-220 (Piotrkow Trybunalski, 3 km)</t>
+          <t>grid node -- PL15-400 (Bydgoszcz, 10 km)</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -807,16 +807,16 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>e_Bialystok_POL</t>
+          <t>e_Mikolow_POL</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>grid node -- PL17-400 (Bialystok, 26 km)</t>
+          <t>grid node -- way/183945016-220 (Katowice, 19 km)</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -850,16 +850,16 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>e_Bydgoszcz_POL</t>
+          <t>e_Olsztyn_POL</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>grid node -- PL15-400 (Bydgoszcz, 10 km)</t>
+          <t>grid node -- way/101915790-220 (Olsztyn, 4 km)</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -893,16 +893,16 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>e_Olsztyn_POL</t>
+          <t>e_Sosnowiec_POL</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>grid node -- way/101915790-220 (Olsztyn, 4 km)</t>
+          <t>grid node -- way/133537926-220 (Katowice, 22 km)</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -933,16 +933,16 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>e_Wloclawek_POL</t>
+          <t>e_Rybnik_POL</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>grid node -- way/245964556-220 (Wloclawek, 10 km)</t>
+          <t>grid node -- way/139452056-400 (Gliwice, 20 km)</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -976,12 +976,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>e_Pulawy_POL</t>
+          <t>e_Swidnik_POL</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>grid node -- way/88544449-220 (Lublin, 46 km)</t>
+          <t>grid node -- way/170249563-220 (Lublin, 6 km)</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -1013,27 +1013,27 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>e_Police_POL</t>
+          <t>e_Wloclawek_POL</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>grid node -- way/165763717-220 (Szczecin, 15 km)</t>
+          <t>grid node -- way/245964556-220 (Wloclawek, 10 km)</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>e_Radomsko_POL</t>
+          <t>e_KamienPomorski_POL</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>grid node -- way/171917072-400 (Czestochowa, 41 km)</t>
+          <t>grid node -- way/165763717-220 (Szczecin, 15 km)</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1052,12 +1052,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>e_Debica_POL</t>
+          <t>e_Rzeszow_POL</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>grid node -- way/198635989-220 (Rzeszow, 6 km)</t>
+          <t>grid node -- way/215282393-400 (Rzeszow, 20 km)</t>
         </is>
       </c>
       <c r="D19" t="n">

</xml_diff>

<commit_message>
Revert "update co2 comm geo"
This reverts commit 998511f295c5e8dcc11fce12e114e7e68d742254.
</commit_message>
<xml_diff>
--- a/VerveStacks_POL_grids_kan50/SubRES_Tmpl/SubRES_Data_Centers_Trans.xlsx
+++ b/VerveStacks_POL_grids_kan50/SubRES_Tmpl/SubRES_Data_Centers_Trans.xlsx
@@ -537,7 +537,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>e_Zabki_POL</t>
+          <t>e_Warsaw_POL</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -560,19 +560,19 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>e_Giszowiec_POL</t>
+          <t>e_Sosnowiec_POL</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>grid node -- PL55-220 (Katowice, 8 km)</t>
+          <t>grid node -- way/183945016-220 (Katowice, 19 km)</t>
         </is>
       </c>
       <c r="C3" t="n">
         <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>327</v>
+        <v>321</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -593,7 +593,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>e_Swarzedz_POL</t>
+          <t>e_Poznan_POL</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -629,7 +629,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>grid node -- way/189501431-400 (Krakow, 13 km)</t>
+          <t>grid node -- way/87667718-220 (Krakow, 12 km)</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -673,7 +673,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>e_Rumia_POL</t>
+          <t>e_Gdansk_POL</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -688,12 +688,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>e_Otwock_POL</t>
+          <t>e_Lomza_POL</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>grid node -- PL26-400 (Warsaw, 53 km)</t>
+          <t>grid node -- way/121656686-220 (Lomza, 31 km)</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -703,12 +703,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>e_PiotrkowTrybunalsk_POL</t>
+          <t>e_Katowice_POL</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>grid node -- way/293484891-400 (Piotrkow Trybunalski, 26 km)</t>
+          <t>grid node -- way/40946790-220 (Katowice, 19 km)</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -718,16 +718,16 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>e_Bialystok_POL</t>
+          <t>e_Gliwice_POL</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>grid node -- PL17-400 (Bialystok, 26 km)</t>
+          <t>grid node -- way/293489607-400 (Katowice, 21 km)</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -743,16 +743,16 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>e_Torun_POL</t>
+          <t>e_PiotrkowTrybunalsk_POL</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>grid node -- PL15-400 (Bydgoszcz, 10 km)</t>
+          <t>grid node -- way/170316833-220 (Piotrkow Trybunalski, 3 km)</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -807,16 +807,16 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>e_Mikolow_POL</t>
+          <t>e_Bialystok_POL</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>grid node -- way/183945016-220 (Katowice, 19 km)</t>
+          <t>grid node -- PL17-400 (Bialystok, 26 km)</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -850,16 +850,16 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>e_Olsztyn_POL</t>
+          <t>e_Bydgoszcz_POL</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>grid node -- way/101915790-220 (Olsztyn, 4 km)</t>
+          <t>grid node -- PL15-400 (Bydgoszcz, 10 km)</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -893,16 +893,16 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>e_Sosnowiec_POL</t>
+          <t>e_Olsztyn_POL</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>grid node -- way/133537926-220 (Katowice, 22 km)</t>
+          <t>grid node -- way/101915790-220 (Olsztyn, 4 km)</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -933,16 +933,16 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>e_Rybnik_POL</t>
+          <t>e_Wloclawek_POL</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>grid node -- way/139452056-400 (Gliwice, 20 km)</t>
+          <t>grid node -- way/245964556-220 (Wloclawek, 10 km)</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -976,12 +976,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>e_Swidnik_POL</t>
+          <t>e_Pulawy_POL</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>grid node -- way/170249563-220 (Lublin, 6 km)</t>
+          <t>grid node -- way/88544449-220 (Lublin, 46 km)</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -1013,27 +1013,27 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>e_Wloclawek_POL</t>
+          <t>e_Police_POL</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>grid node -- way/245964556-220 (Wloclawek, 10 km)</t>
+          <t>grid node -- way/165763717-220 (Szczecin, 15 km)</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>e_KamienPomorski_POL</t>
+          <t>e_Radomsko_POL</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>grid node -- way/165763717-220 (Szczecin, 15 km)</t>
+          <t>grid node -- way/171917072-400 (Czestochowa, 41 km)</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1052,12 +1052,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>e_Rzeszow_POL</t>
+          <t>e_Debica_POL</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>grid node -- way/215282393-400 (Rzeszow, 20 km)</t>
+          <t>grid node -- way/198635989-220 (Rzeszow, 6 km)</t>
         </is>
       </c>
       <c r="D19" t="n">

</xml_diff>

<commit_message>
Updated POL_grids_kan50 model - 2026-10-03 14:34
</commit_message>
<xml_diff>
--- a/VerveStacks_POL_grids_kan50/SubRES_Tmpl/SubRES_Data_Centers_Trans.xlsx
+++ b/VerveStacks_POL_grids_kan50/SubRES_Tmpl/SubRES_Data_Centers_Trans.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="DC details" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DC details" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>

</xml_diff>